<commit_message>
chore(PDG-59): tidy preNormalization/sourceConfig rule files
Trim a trailing space in the OFAC-NON-SDN entity_type cell (preNormalization) so the rule scopes correctly; sourceConfig is an Excel re-save with no content change. Full unit suite green.
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CA3EC3-4E3A-459D-99A9-137BC8347182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201EBBA2-FEFA-4D3A-9C60-E91F6610ACD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1780" yWindow="1780" windowWidth="15680" windowHeight="9430" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="15680" windowHeight="9430" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(PDG-90): onboard CANADA_CONSOLIDATED_SANCTIONS watchlist
Global Affairs Canada consolidated autonomous sanctions XML (5,707 records). Composite id from regime+schedule+item; entity type stamped from filled columns; pre-norm keeps English regime/title, maps ship types to picklist, splits aliases. Adds Ro-Ro Vessel, Heavy Lift Vessel, Floating Storage Unit vessel types.

Shared rule-file changes: mapping.xlsx Group case typo (rows 281-282) fixed, restoring VesselDetails for vessel lists incl. UKSL (0 -> 657); DatasetCategory PEP (Politically Exposed Person) -> PEP for DILG/COMELEC/PH-HOUSE/CIA and Crime+Sanctions -> Sanctions for ATC individuals and US-STATE, with golden tests updated.
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E58E1A2B-0E34-46D7-9398-658663CF49DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99DC7F97-8BC5-44CD-8192-7883AA9D13C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>source</t>
   </si>
@@ -125,6 +125,12 @@
   </si>
   <si>
     <t>unique_id</t>
+  </si>
+  <si>
+    <t>CANADA_CONSOLIDATED_SANCTIONS</t>
+  </si>
+  <si>
+    <t>entity_type</t>
   </si>
 </sst>
 </file>
@@ -501,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC009C7E-7FED-434A-80FD-C4CDDA6E12F9}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="21.58203125" customWidth="1"/>
@@ -639,6 +645,17 @@
         <v>29</v>
       </c>
     </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add BIS denied persons watchlist source
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99DC7F97-8BC5-44CD-8192-7883AA9D13C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C26536-3536-4734-8F7B-B5C864E733B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
+    <workbookView xWindow="380" yWindow="1950" windowWidth="13550" windowHeight="9670" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>source</t>
   </si>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>entity_type</t>
+  </si>
+  <si>
+    <t>BIS-DPL</t>
+  </si>
+  <si>
+    <t>source_record_id</t>
   </si>
 </sst>
 </file>
@@ -185,13 +191,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -507,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC009C7E-7FED-434A-80FD-C4CDDA6E12F9}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="21.58203125" customWidth="1"/>
@@ -656,6 +665,17 @@
         <v>29</v>
       </c>
     </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add BIS Unverified List and refine entity classification
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C26536-3536-4734-8F7B-B5C864E733B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B6BE7E-AFD4-4F05-9881-E0535E73825D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="1950" windowWidth="13550" windowHeight="9670" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
   <si>
     <t>source</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>source_record_id</t>
+  </si>
+  <si>
+    <t>BIS_UNVERIFIED_LIST</t>
   </si>
 </sst>
 </file>
@@ -516,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC009C7E-7FED-434A-80FD-C4CDDA6E12F9}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="21.58203125" customWidth="1"/>
@@ -676,6 +679,17 @@
         <v>33</v>
       </c>
     </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add BIS Military End-User List
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B6BE7E-AFD4-4F05-9881-E0535E73825D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8139F7F6-0F3B-4C3B-A002-C810F83A1417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
+    <workbookView xWindow="2540" yWindow="1610" windowWidth="13550" windowHeight="9670" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>source</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>BIS_UNVERIFIED_LIST</t>
+  </si>
+  <si>
+    <t>BIS_MILITARY_END_USER_LIST</t>
   </si>
 </sst>
 </file>
@@ -519,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC009C7E-7FED-434A-80FD-C4CDDA6E12F9}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="21.58203125" customWidth="1"/>
@@ -690,6 +693,17 @@
         <v>33</v>
       </c>
     </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(PDG-89): onboard EBRD_INELIGIBLE_ENTITIES watchlist
Collect the EBRD ineligible entities list from the JSON endpoint behind
the site (filterlistservlet, paged by currentPage) with the existing API
collector. The CSV export is not used: unquoted commas break parsing and
quoted names come out mangled.

- Record id: composite hash of title, nationality, address, grounds and
  the debarment start/end dates.
- Entity type routed from projectNoticeType via sourceConfig + enum.
- Names/aliases split from title and subtitle; native-script names go
  to Names[] as Original Script; Mr/Ms/Dr titles and the "and any entity
  controlled" tail removed from individual names.
- Ongoing/Indefinite end dates mapped to Measures[].Duration.
- Reasons mapped to additionalInfo Offense, grounds to Measures[].Note.
- Add a 50-record sample to the conformance and golden tests.

mapping.xlsx also carries pending OFAC-SDN, OFAC-NON-SDN and
US-STATE-TERRORIST-EXCLUSION mapping edits made before this branch.
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8139F7F6-0F3B-4C3B-A002-C810F83A1417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44861B9D-DDC6-4590-97CF-C870720347C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2540" yWindow="1610" windowWidth="13550" windowHeight="9670" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>source</t>
   </si>
@@ -143,6 +143,12 @@
   </si>
   <si>
     <t>BIS_MILITARY_END_USER_LIST</t>
+  </si>
+  <si>
+    <t>EBRD_INELIGIBLE_ENTITIES</t>
+  </si>
+  <si>
+    <t>projectNoticeType</t>
   </si>
 </sst>
 </file>
@@ -197,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -207,6 +213,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -522,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC009C7E-7FED-434A-80FD-C4CDDA6E12F9}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="21.58203125" customWidth="1"/>
@@ -704,6 +713,17 @@
         <v>33</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="25">
+      <c r="A17" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add Philippine Supreme Court incumbent justices watchlist
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6170F7C-3DE9-4265-8C45-1797FDEBB9AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8292174-5880-4C75-844E-E9F68FE349F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3340" yWindow="1610" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
   <si>
     <t>source</t>
   </si>
@@ -143,6 +143,9 @@
   </si>
   <si>
     <t>Entity</t>
+  </si>
+  <si>
+    <t>SC_PH_INCUMBENT_JUSTICES</t>
   </si>
 </sst>
 </file>
@@ -517,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="21.58203125" customWidth="1"/>
@@ -732,6 +735,17 @@
         <v>33</v>
       </c>
     </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add SEC PAUSE watchlist with pagination, profile extraction and mapping
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E28027-EF6E-44A0-80FD-91490E3E88D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4C7858-F056-4524-8E1E-D9DA5BF3B4BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
   <si>
     <t>source</t>
   </si>
@@ -152,13 +152,16 @@
   </si>
   <si>
     <t>SC_PH_INCUMBENT_JUSTICES</t>
+  </si>
+  <si>
+    <t>SEC_US_PAUSE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -174,24 +177,26 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Unicode MS"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -206,20 +211,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,26 +521,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.58203125" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" customWidth="1"/>
     <col min="3" max="3" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -556,7 +551,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -565,7 +560,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -576,192 +571,208 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="31">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="3" t="s">
+      <c r="C14" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="3" t="s">
+      <c r="C15" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="25">
-      <c r="A17" s="6" t="s">
+      <c r="C16" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="25">
-      <c r="A18" s="6" t="s">
+      <c r="C17" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
+      <c r="C18" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
+      <c r="C19" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
+      <c r="C20" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C21" t="s">
-        <v>33</v>
-      </c>
+      <c r="C21" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(PDG-98,PDG-119): add HKPF source and normalization rules
Add both HKPF list mappings and normalization rules. Preserve the intentional SEC-US and SEC_US_PAUSE picklist removals and the existing BSP and Crimestoppers workbook edits.
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0879DF01-4F0B-4B7F-9B44-0B6E8FC86385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4DB883C-2C9B-4B17-B033-710FA9C86BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2330" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="48">
   <si>
     <t>source</t>
   </si>
@@ -158,6 +158,12 @@
   </si>
   <si>
     <t>CRIMESTOPPERS_UK_MOST_WANTED</t>
+  </si>
+  <si>
+    <t>HKPF_WANTED_PERSONS_NATIONAL_SECURITY</t>
+  </si>
+  <si>
+    <t>HKPF_WANTED_PERSONS_WITH_REWARD_NOTICES</t>
   </si>
 </sst>
 </file>
@@ -530,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="30.58203125" customWidth="1"/>
@@ -789,6 +795,28 @@
         <v>33</v>
       </c>
     </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>